<commit_message>
feat: integrar foro en blog, corregir banners, mapas y unificar nombres institucionales
</commit_message>
<xml_diff>
--- a/MT Colombia _ Accesos Digitales (1) (1).xlsx
+++ b/MT Colombia _ Accesos Digitales (1) (1).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javir\Documents\Caro centro mt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javir\Documents\DEVs\web_centro_mt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9242F6E3-5E35-4370-B9E3-B33F3C0BAA3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30C8706E-8CD3-4DC9-A748-3E1FEA54FC3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -95,7 +95,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -141,6 +141,13 @@
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -196,10 +203,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -222,8 +230,12 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -445,7 +457,8 @@
   <cols>
     <col min="1" max="2" width="17.42578125" customWidth="1"/>
     <col min="3" max="3" width="30.42578125" customWidth="1"/>
-    <col min="4" max="7" width="17.42578125" customWidth="1"/>
+    <col min="4" max="4" width="33.28515625" customWidth="1"/>
+    <col min="5" max="7" width="17.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="19.5" x14ac:dyDescent="0.2">
@@ -528,7 +541,7 @@
       <c r="Y2" s="2"/>
       <c r="Z2" s="2"/>
     </row>
-    <row r="3" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -576,7 +589,7 @@
       <c r="C4" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="8" t="s">
         <v>19</v>
       </c>
       <c r="E4" s="2" t="s">
@@ -647,7 +660,7 @@
         <v>22</v>
       </c>
       <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
+      <c r="C6" s="6"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -28515,6 +28528,7 @@
     <hyperlink ref="C3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="C4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
     <hyperlink ref="C5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="D4" r:id="rId5" xr:uid="{53316B33-9385-477B-85C1-03B6523F414B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>